<commit_message>
docs & feat: refactored AIVisualize into 4 sections, AIOptimize into 2 tracks, and added 4 new generators
</commit_message>
<xml_diff>
--- a/_context/AEO_TOOL_MAPPING_V1.xlsx
+++ b/_context/AEO_TOOL_MAPPING_V1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MyApps\aeo-audit-tool-v2\.gemini\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MyApps\aeo-audit-tool-v3\_context\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE6F5BEC-79C8-48A3-85A9-F47A341050C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A51111A1-CD1F-4288-80F2-FA0582BBCCD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{6073F0D8-4F6F-4048-AC8C-2714F136D76E}"/>
   </bookViews>
@@ -17,7 +17,6 @@
     <sheet name="Glossary" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -41,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1774" uniqueCount="286">
   <si>
     <t>AISocialize</t>
   </si>
@@ -896,6 +895,21 @@
   </si>
   <si>
     <t>Authoritativeness analysis:  authority Links(Valid per page)</t>
+  </si>
+  <si>
+    <t>Site</t>
+  </si>
+  <si>
+    <t>page</t>
+  </si>
+  <si>
+    <t>Page</t>
+  </si>
+  <si>
+    <t>Per Page/Site/Post</t>
+  </si>
+  <si>
+    <t>Post</t>
   </si>
 </sst>
 </file>
@@ -960,7 +974,10 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="19">
+  <dxfs count="20">
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1032,35 +1049,36 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FD337438-C06E-4F50-BBED-8980A160B1E2}" name="Table1" displayName="Table1" ref="A1:J115" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
-  <autoFilter ref="A1:J115" xr:uid="{FD337438-C06E-4F50-BBED-8980A160B1E2}"/>
-  <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{EA71DEFB-ED09-4AF2-B003-CFBC5B42A87C}" name="Type" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{84601B03-3507-43FC-A95E-7037795D6DD0}" name="Diagnostic Metric" dataDxfId="10"/>
-    <tableColumn id="6" xr3:uid="{8BC27A12-C4F3-4C59-8694-55178052D543}" name="Description" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{7184A817-11AA-4061-B4A6-9A32F9B2F1E1}" name="AIVisualize Free" dataDxfId="8"/>
-    <tableColumn id="7" xr3:uid="{3D62F163-5F2C-4A0D-AF77-38EBA86A3320}" name="AIV Pro" dataDxfId="7"/>
-    <tableColumn id="8" xr3:uid="{EE7ACD9C-FF77-4A7A-846D-CE90F0199399}" name="AIV Enteprise" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{B61E96FF-F86A-452D-838A-DF1579880F1E}" name="AIOptimize Free" dataDxfId="5"/>
-    <tableColumn id="10" xr3:uid="{438EC34F-0CC0-4E3C-9D3D-B7C9E6959881}" name="AIO Pro" dataDxfId="4"/>
-    <tableColumn id="9" xr3:uid="{F532B431-FF0C-49B8-8390-4E93C0392614}" name="AIO Ent" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{10CEA263-1AF0-4D56-A841-D5503ADE949B}" name="AISocialize" dataDxfId="2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FD337438-C06E-4F50-BBED-8980A160B1E2}" name="Table1" displayName="Table1" ref="A1:K115" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
+  <autoFilter ref="A1:K115" xr:uid="{FD337438-C06E-4F50-BBED-8980A160B1E2}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{EA71DEFB-ED09-4AF2-B003-CFBC5B42A87C}" name="Type" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{84601B03-3507-43FC-A95E-7037795D6DD0}" name="Diagnostic Metric" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{8BC27A12-C4F3-4C59-8694-55178052D543}" name="Description" dataDxfId="15"/>
+    <tableColumn id="11" xr3:uid="{C236DB6A-54A9-4484-A89C-DE7FD4AA9DB9}" name="Per Page/Site/Post" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{7184A817-11AA-4061-B4A6-9A32F9B2F1E1}" name="AIVisualize Free" dataDxfId="14"/>
+    <tableColumn id="7" xr3:uid="{3D62F163-5F2C-4A0D-AF77-38EBA86A3320}" name="AIV Pro" dataDxfId="13"/>
+    <tableColumn id="8" xr3:uid="{EE7ACD9C-FF77-4A7A-846D-CE90F0199399}" name="AIV Enteprise" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{B61E96FF-F86A-452D-838A-DF1579880F1E}" name="AIOptimize Free" dataDxfId="11"/>
+    <tableColumn id="10" xr3:uid="{438EC34F-0CC0-4E3C-9D3D-B7C9E6959881}" name="AIO Pro" dataDxfId="10"/>
+    <tableColumn id="9" xr3:uid="{F532B431-FF0C-49B8-8390-4E93C0392614}" name="AIO Ent" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{10CEA263-1AF0-4D56-A841-D5503ADE949B}" name="AISocialize" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8EB6CC0A-48B2-4B40-A13F-845A167F3B8D}" name="Table2" displayName="Table2" ref="A1:G10" totalsRowShown="0" dataDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8EB6CC0A-48B2-4B40-A13F-845A167F3B8D}" name="Table2" displayName="Table2" ref="A1:G10" totalsRowShown="0" dataDxfId="7">
   <autoFilter ref="A1:G10" xr:uid="{8EB6CC0A-48B2-4B40-A13F-845A167F3B8D}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{2CE08055-56BC-461F-A131-8C9DB0A2D104}" name="File"/>
-    <tableColumn id="2" xr3:uid="{F1650DA2-CC80-497B-A8DA-C7EC6A18C345}" name="What is is" dataDxfId="18"/>
-    <tableColumn id="3" xr3:uid="{5AF922AD-7BB8-409F-8275-8F6E09A556E2}" name="What uses it" dataDxfId="17"/>
-    <tableColumn id="4" xr3:uid="{5B21E9F7-F1BD-473A-8186-4CB692DF29C7}" name="How is it used?" dataDxfId="16"/>
-    <tableColumn id="5" xr3:uid="{187AAE0D-A7EE-414E-84C7-C67D02CE41B4}" name="What is it used for?" dataDxfId="15"/>
-    <tableColumn id="6" xr3:uid="{65BC5AE4-144A-4D27-BAA1-54746E680FAE}" name="Where should it be available" dataDxfId="14"/>
-    <tableColumn id="7" xr3:uid="{775AF47D-6201-4DB5-A7DF-2EE501E97B47}" name="template" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{F1650DA2-CC80-497B-A8DA-C7EC6A18C345}" name="What is is" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{5AF922AD-7BB8-409F-8275-8F6E09A556E2}" name="What uses it" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{5B21E9F7-F1BD-473A-8186-4CB692DF29C7}" name="How is it used?" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{187AAE0D-A7EE-414E-84C7-C67D02CE41B4}" name="What is it used for?" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{65BC5AE4-144A-4D27-BAA1-54746E680FAE}" name="Where should it be available" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{775AF47D-6201-4DB5-A7DF-2EE501E97B47}" name="template" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1383,19 +1401,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55A4A3A0-5979-416B-A6BF-400E246F3969}">
-  <dimension ref="A1:J115"/>
+  <dimension ref="A1:K115"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="43.21875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="36.21875" style="1" customWidth="1"/>
-    <col min="4" max="6" width="16.6640625" style="1" customWidth="1"/>
-    <col min="7" max="9" width="16" style="1" customWidth="1"/>
-    <col min="10" max="10" width="17.5546875" style="1" customWidth="1"/>
-    <col min="11" max="16384" width="8.88671875" style="1"/>
+    <col min="3" max="4" width="36.21875" style="1" customWidth="1"/>
+    <col min="5" max="7" width="16.6640625" style="1" customWidth="1"/>
+    <col min="8" max="10" width="16" style="1" customWidth="1"/>
+    <col min="11" max="11" width="17.5546875" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>25</v>
       </c>
@@ -1406,28 +1424,31 @@
         <v>52</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>26</v>
       </c>
@@ -1435,7 +1456,7 @@
         <v>2</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>145</v>
+        <v>281</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>145</v>
@@ -1452,8 +1473,11 @@
       <c r="I2" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J2" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>26</v>
       </c>
@@ -1461,7 +1485,7 @@
         <v>3</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>145</v>
+        <v>281</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>145</v>
@@ -1478,8 +1502,11 @@
       <c r="I3" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="J3" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>26</v>
       </c>
@@ -1487,11 +1514,11 @@
         <v>4</v>
       </c>
       <c r="D4" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>145</v>
-      </c>
       <c r="F4" s="1" t="s">
         <v>145</v>
       </c>
@@ -1504,8 +1531,11 @@
       <c r="I4" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="J4" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>26</v>
       </c>
@@ -1513,11 +1543,11 @@
         <v>5</v>
       </c>
       <c r="D5" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>145</v>
-      </c>
       <c r="F5" s="1" t="s">
         <v>145</v>
       </c>
@@ -1530,8 +1560,11 @@
       <c r="I5" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J5" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>26</v>
       </c>
@@ -1539,7 +1572,7 @@
         <v>132</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>145</v>
+        <v>281</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>145</v>
@@ -1556,8 +1589,11 @@
       <c r="I6" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="J6" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>26</v>
       </c>
@@ -1565,7 +1601,7 @@
         <v>47</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>232</v>
+        <v>281</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>232</v>
@@ -1574,7 +1610,7 @@
         <v>232</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>145</v>
+        <v>232</v>
       </c>
       <c r="H7" s="1" t="s">
         <v>145</v>
@@ -1582,8 +1618,11 @@
       <c r="I7" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="J7" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>26</v>
       </c>
@@ -1594,7 +1633,7 @@
         <v>192</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>145</v>
+        <v>281</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>145</v>
@@ -1602,8 +1641,11 @@
       <c r="F8" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="G8" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>218</v>
       </c>
@@ -1614,7 +1656,7 @@
         <v>219</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>145</v>
+        <v>282</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>145</v>
@@ -1622,8 +1664,11 @@
       <c r="F9" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="G9" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>218</v>
       </c>
@@ -1634,7 +1679,7 @@
         <v>220</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>232</v>
+        <v>283</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>232</v>
@@ -1646,13 +1691,16 @@
         <v>232</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>145</v>
+        <v>232</v>
       </c>
       <c r="I10" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="J10" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>218</v>
       </c>
@@ -1663,7 +1711,7 @@
         <v>223</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>232</v>
+        <v>283</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>232</v>
@@ -1675,13 +1723,16 @@
         <v>232</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>145</v>
+        <v>232</v>
       </c>
       <c r="I11" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J11" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>27</v>
       </c>
@@ -1689,13 +1740,16 @@
         <v>6</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+        <v>281</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>27</v>
       </c>
@@ -1703,7 +1757,7 @@
         <v>7</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>232</v>
+        <v>281</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>232</v>
@@ -1715,13 +1769,16 @@
         <v>232</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>145</v>
+        <v>232</v>
       </c>
       <c r="I13" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="J13" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>28</v>
       </c>
@@ -1729,7 +1786,7 @@
         <v>8</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>232</v>
+        <v>281</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>232</v>
@@ -1741,13 +1798,16 @@
         <v>232</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>145</v>
+        <v>232</v>
       </c>
       <c r="I14" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="15" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="J14" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>28</v>
       </c>
@@ -1755,7 +1815,7 @@
         <v>9</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>232</v>
+        <v>281</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>232</v>
@@ -1767,13 +1827,16 @@
         <v>232</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>145</v>
+        <v>232</v>
       </c>
       <c r="I15" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="J15" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>28</v>
       </c>
@@ -1781,7 +1844,7 @@
         <v>10</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>232</v>
+        <v>281</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>232</v>
@@ -1793,13 +1856,16 @@
         <v>232</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>145</v>
+        <v>232</v>
       </c>
       <c r="I16" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J16" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>29</v>
       </c>
@@ -1807,13 +1873,16 @@
         <v>30</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="J17" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+        <v>283</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="K17" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>29</v>
       </c>
@@ -1821,19 +1890,22 @@
         <v>31</v>
       </c>
       <c r="D18" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="E18" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="E18" s="1" t="s">
-        <v>145</v>
-      </c>
       <c r="F18" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="J18" s="1" t="s">
+      <c r="G18" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="K18" s="1" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>29</v>
       </c>
@@ -1841,7 +1913,7 @@
         <v>32</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>234</v>
+        <v>283</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>234</v>
@@ -1850,7 +1922,7 @@
         <v>234</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>145</v>
+        <v>234</v>
       </c>
       <c r="H19" s="1" t="s">
         <v>145</v>
@@ -1859,10 +1931,13 @@
         <v>145</v>
       </c>
       <c r="J19" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="K19" s="1" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>17</v>
       </c>
@@ -1870,7 +1945,7 @@
         <v>33</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>145</v>
+        <v>281</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>145</v>
@@ -1878,11 +1953,14 @@
       <c r="F20" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="J20" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="G20" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="K20" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>17</v>
       </c>
@@ -1890,7 +1968,7 @@
         <v>34</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>145</v>
+        <v>281</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>145</v>
@@ -1898,11 +1976,14 @@
       <c r="F21" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="J21" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="G21" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="K21" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>17</v>
       </c>
@@ -1910,7 +1991,7 @@
         <v>193</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>145</v>
+        <v>281</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>145</v>
@@ -1918,11 +1999,14 @@
       <c r="F22" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="J22" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="G22" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="K22" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>17</v>
       </c>
@@ -1930,7 +2014,7 @@
         <v>35</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>232</v>
+        <v>281</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>232</v>
@@ -1942,16 +2026,19 @@
         <v>232</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>145</v>
+        <v>232</v>
       </c>
       <c r="I23" s="1" t="s">
         <v>145</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+        <v>145</v>
+      </c>
+      <c r="K23" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>17</v>
       </c>
@@ -1959,7 +2046,7 @@
         <v>36</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>232</v>
+        <v>281</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>232</v>
@@ -1971,49 +2058,61 @@
         <v>232</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>145</v>
+        <v>232</v>
       </c>
       <c r="I24" s="1" t="s">
         <v>145</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+        <v>145</v>
+      </c>
+      <c r="K24" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="J25" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D25" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="K25" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="J26" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="D26" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="K26" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="J27" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="D27" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="K27" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>18</v>
       </c>
@@ -2021,7 +2120,7 @@
         <v>43</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>145</v>
+        <v>281</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>145</v>
@@ -2029,8 +2128,11 @@
       <c r="F28" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="G28" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>18</v>
       </c>
@@ -2038,7 +2140,7 @@
         <v>44</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>145</v>
+        <v>281</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>145</v>
@@ -2046,8 +2148,11 @@
       <c r="F29" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="G29" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>18</v>
       </c>
@@ -2055,7 +2160,7 @@
         <v>46</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>145</v>
+        <v>281</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>145</v>
@@ -2063,8 +2168,11 @@
       <c r="F30" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="G30" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>18</v>
       </c>
@@ -2072,7 +2180,7 @@
         <v>146</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>145</v>
+        <v>281</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>145</v>
@@ -2080,8 +2188,11 @@
       <c r="F31" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="32" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="G31" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>18</v>
       </c>
@@ -2089,21 +2200,24 @@
         <v>194</v>
       </c>
       <c r="D32" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="E32" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="E32" s="1" t="s">
-        <v>145</v>
-      </c>
       <c r="F32" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G32" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B33" s="1" t="s">
         <v>45</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>145</v>
+        <v>281</v>
       </c>
       <c r="E33" s="1" t="s">
         <v>145</v>
@@ -2111,8 +2225,11 @@
       <c r="F33" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="34" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="G33" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
         <v>18</v>
       </c>
@@ -2123,7 +2240,7 @@
         <v>238</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>232</v>
+        <v>281</v>
       </c>
       <c r="E34" s="1" t="s">
         <v>232</v>
@@ -2132,16 +2249,19 @@
         <v>232</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>145</v>
+        <v>232</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>237</v>
+        <v>145</v>
       </c>
       <c r="I34" s="1" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="35" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="J34" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>55</v>
       </c>
@@ -2152,7 +2272,7 @@
         <v>239</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>232</v>
+        <v>281</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>232</v>
@@ -2161,16 +2281,19 @@
         <v>232</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>145</v>
+        <v>232</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>237</v>
+        <v>145</v>
       </c>
       <c r="I35" s="1" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J35" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
         <v>185</v>
       </c>
@@ -2178,7 +2301,7 @@
         <v>186</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>145</v>
+        <v>281</v>
       </c>
       <c r="E36" s="1" t="s">
         <v>145</v>
@@ -2186,8 +2309,11 @@
       <c r="F36" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="37" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="G36" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
         <v>189</v>
       </c>
@@ -2195,7 +2321,7 @@
         <v>190</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>145</v>
+        <v>281</v>
       </c>
       <c r="E37" s="1" t="s">
         <v>145</v>
@@ -2203,8 +2329,11 @@
       <c r="F37" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="38" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="G37" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
         <v>187</v>
       </c>
@@ -2212,7 +2341,7 @@
         <v>188</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>145</v>
+        <v>281</v>
       </c>
       <c r="E38" s="1" t="s">
         <v>145</v>
@@ -2220,8 +2349,11 @@
       <c r="F38" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G38" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
         <v>22</v>
       </c>
@@ -2229,7 +2361,7 @@
         <v>37</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>145</v>
+        <v>281</v>
       </c>
       <c r="E39" s="1" t="s">
         <v>145</v>
@@ -2237,8 +2369,11 @@
       <c r="F39" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="40" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="G39" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
         <v>22</v>
       </c>
@@ -2246,16 +2381,19 @@
         <v>195</v>
       </c>
       <c r="D40" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="E40" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="E40" s="1" t="s">
-        <v>145</v>
-      </c>
       <c r="F40" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="41" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="G40" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
         <v>22</v>
       </c>
@@ -2265,17 +2403,20 @@
       <c r="C41" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="G41" s="1" t="s">
-        <v>145</v>
+      <c r="D41" s="1" t="s">
+        <v>281</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>237</v>
+        <v>145</v>
       </c>
       <c r="I41" s="1" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J41" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
         <v>149</v>
       </c>
@@ -2283,7 +2424,7 @@
         <v>148</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>145</v>
+        <v>281</v>
       </c>
       <c r="E42" s="1" t="s">
         <v>145</v>
@@ -2291,8 +2432,11 @@
       <c r="F42" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G42" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
         <v>183</v>
       </c>
@@ -2300,7 +2444,7 @@
         <v>184</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>145</v>
+        <v>281</v>
       </c>
       <c r="E43" s="1" t="s">
         <v>145</v>
@@ -2308,8 +2452,11 @@
       <c r="F43" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="44" spans="1:9" ht="158.4" x14ac:dyDescent="0.3">
+      <c r="G43" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
         <v>39</v>
       </c>
@@ -2320,7 +2467,7 @@
         <v>68</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>145</v>
+        <v>281</v>
       </c>
       <c r="E44" s="1" t="s">
         <v>145</v>
@@ -2328,8 +2475,11 @@
       <c r="F44" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="45" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="G44" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
         <v>39</v>
       </c>
@@ -2337,16 +2487,19 @@
         <v>196</v>
       </c>
       <c r="D45" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="E45" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="E45" s="1" t="s">
-        <v>145</v>
-      </c>
       <c r="F45" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="46" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="G45" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
         <v>39</v>
       </c>
@@ -2357,7 +2510,7 @@
         <v>241</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>232</v>
+        <v>281</v>
       </c>
       <c r="E46" s="1" t="s">
         <v>232</v>
@@ -2366,16 +2519,19 @@
         <v>232</v>
       </c>
       <c r="G46" s="1" t="s">
-        <v>145</v>
+        <v>232</v>
       </c>
       <c r="H46" s="1" t="s">
-        <v>237</v>
+        <v>145</v>
       </c>
       <c r="I46" s="1" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="47" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="J46" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
         <v>39</v>
       </c>
@@ -2386,7 +2542,7 @@
         <v>242</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>232</v>
+        <v>281</v>
       </c>
       <c r="E47" s="1" t="s">
         <v>232</v>
@@ -2395,16 +2551,19 @@
         <v>232</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>145</v>
+        <v>232</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>237</v>
+        <v>145</v>
       </c>
       <c r="I47" s="1" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J47" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
         <v>150</v>
       </c>
@@ -2412,7 +2571,7 @@
         <v>151</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>145</v>
+        <v>281</v>
       </c>
       <c r="E48" s="1" t="s">
         <v>145</v>
@@ -2420,8 +2579,11 @@
       <c r="F48" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="49" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="G48" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
         <v>177</v>
       </c>
@@ -2429,7 +2591,7 @@
         <v>178</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>145</v>
+        <v>281</v>
       </c>
       <c r="E49" s="1" t="s">
         <v>145</v>
@@ -2437,8 +2599,11 @@
       <c r="F49" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="G49" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
         <v>23</v>
       </c>
@@ -2446,7 +2611,7 @@
         <v>42</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>145</v>
+        <v>281</v>
       </c>
       <c r="E50" s="1" t="s">
         <v>145</v>
@@ -2454,11 +2619,14 @@
       <c r="F50" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="J50" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="G50" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="K50" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
         <v>23</v>
       </c>
@@ -2466,19 +2634,22 @@
         <v>197</v>
       </c>
       <c r="D51" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="E51" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="E51" s="1" t="s">
-        <v>145</v>
-      </c>
       <c r="F51" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="J51" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G51" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="K51" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
         <v>23</v>
       </c>
@@ -2489,7 +2660,7 @@
         <v>243</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>232</v>
+        <v>281</v>
       </c>
       <c r="E52" s="1" t="s">
         <v>232</v>
@@ -2498,19 +2669,22 @@
         <v>232</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>145</v>
+        <v>232</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>237</v>
+        <v>145</v>
       </c>
       <c r="I52" s="1" t="s">
         <v>237</v>
       </c>
       <c r="J52" s="1" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
+        <v>237</v>
+      </c>
+      <c r="K52" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
         <v>179</v>
       </c>
@@ -2518,7 +2692,7 @@
         <v>180</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>145</v>
+        <v>281</v>
       </c>
       <c r="E53" s="1" t="s">
         <v>145</v>
@@ -2526,11 +2700,14 @@
       <c r="F53" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="J53" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="G53" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="K53" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
         <v>181</v>
       </c>
@@ -2538,7 +2715,7 @@
         <v>182</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>145</v>
+        <v>281</v>
       </c>
       <c r="E54" s="1" t="s">
         <v>145</v>
@@ -2546,11 +2723,14 @@
       <c r="F54" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="J54" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="G54" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="K54" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
         <v>133</v>
       </c>
@@ -2558,7 +2738,7 @@
         <v>175</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>145</v>
+        <v>281</v>
       </c>
       <c r="E55" s="1" t="s">
         <v>145</v>
@@ -2566,8 +2746,11 @@
       <c r="F55" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="56" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="G55" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
         <v>133</v>
       </c>
@@ -2575,16 +2758,19 @@
         <v>176</v>
       </c>
       <c r="D56" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="E56" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="E56" s="1" t="s">
-        <v>145</v>
-      </c>
       <c r="F56" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="57" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="G56" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
         <v>133</v>
       </c>
@@ -2595,7 +2781,7 @@
         <v>213</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>232</v>
+        <v>281</v>
       </c>
       <c r="E57" s="1" t="s">
         <v>232</v>
@@ -2604,16 +2790,19 @@
         <v>232</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>145</v>
+        <v>232</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>237</v>
+        <v>145</v>
       </c>
       <c r="I57" s="1" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="58" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="J57" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
         <v>48</v>
       </c>
@@ -2624,16 +2813,19 @@
         <v>54</v>
       </c>
       <c r="D58" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="E58" s="1" t="s">
         <v>272</v>
       </c>
-      <c r="E58" s="1" t="s">
+      <c r="F58" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="F58" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G58" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
         <v>48</v>
       </c>
@@ -2644,7 +2836,7 @@
         <v>53</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>145</v>
+        <v>281</v>
       </c>
       <c r="E59" s="1" t="s">
         <v>145</v>
@@ -2652,8 +2844,11 @@
       <c r="F59" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="G59" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
         <v>51</v>
       </c>
@@ -2661,7 +2856,7 @@
         <v>198</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>145</v>
+        <v>283</v>
       </c>
       <c r="E60" s="1" t="s">
         <v>145</v>
@@ -2669,8 +2864,11 @@
       <c r="F60" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="61" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="G60" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
         <v>51</v>
       </c>
@@ -2678,7 +2876,7 @@
         <v>199</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>145</v>
+        <v>283</v>
       </c>
       <c r="E61" s="1" t="s">
         <v>145</v>
@@ -2686,8 +2884,11 @@
       <c r="F61" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="62" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G61" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
         <v>60</v>
       </c>
@@ -2698,7 +2899,7 @@
         <v>59</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>232</v>
+        <v>283</v>
       </c>
       <c r="E62" s="1" t="s">
         <v>232</v>
@@ -2707,16 +2908,19 @@
         <v>232</v>
       </c>
       <c r="G62" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H62" s="1" t="s">
         <v>244</v>
-      </c>
-      <c r="H62" s="1" t="s">
-        <v>237</v>
       </c>
       <c r="I62" s="1" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="63" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="J62" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
         <v>61</v>
       </c>
@@ -2724,7 +2928,7 @@
         <v>64</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>145</v>
+        <v>283</v>
       </c>
       <c r="E63" s="1" t="s">
         <v>145</v>
@@ -2732,8 +2936,11 @@
       <c r="F63" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="64" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G63" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A64" s="1" t="s">
         <v>61</v>
       </c>
@@ -2741,7 +2948,7 @@
         <v>65</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>232</v>
+        <v>283</v>
       </c>
       <c r="E64" s="1" t="s">
         <v>232</v>
@@ -2750,16 +2957,19 @@
         <v>232</v>
       </c>
       <c r="G64" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H64" s="1" t="s">
         <v>245</v>
-      </c>
-      <c r="H64" s="1" t="s">
-        <v>237</v>
       </c>
       <c r="I64" s="1" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="65" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="J64" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A65" s="1" t="s">
         <v>61</v>
       </c>
@@ -2767,7 +2977,7 @@
         <v>62</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>232</v>
+        <v>283</v>
       </c>
       <c r="E65" s="1" t="s">
         <v>232</v>
@@ -2776,16 +2986,19 @@
         <v>232</v>
       </c>
       <c r="G65" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H65" s="1" t="s">
         <v>245</v>
-      </c>
-      <c r="H65" s="1" t="s">
-        <v>237</v>
       </c>
       <c r="I65" s="1" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="66" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="J65" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A66" s="1" t="s">
         <v>69</v>
       </c>
@@ -2793,7 +3006,7 @@
         <v>70</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>145</v>
+        <v>283</v>
       </c>
       <c r="E66" s="1" t="s">
         <v>145</v>
@@ -2801,11 +3014,14 @@
       <c r="F66" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="J66" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="67" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="G66" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="K66" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A67" s="1" t="s">
         <v>71</v>
       </c>
@@ -2816,10 +3032,13 @@
         <v>247</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="68" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+        <v>283</v>
+      </c>
+      <c r="E67" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A68" s="1" t="s">
         <v>71</v>
       </c>
@@ -2830,16 +3049,19 @@
         <v>73</v>
       </c>
       <c r="D68" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="E68" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="E68" s="1" t="s">
-        <v>145</v>
-      </c>
       <c r="F68" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="69" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="G68" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A69" s="1" t="s">
         <v>74</v>
       </c>
@@ -2847,7 +3069,7 @@
         <v>200</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>145</v>
+        <v>283</v>
       </c>
       <c r="E69" s="1" t="s">
         <v>145</v>
@@ -2855,8 +3077,11 @@
       <c r="F69" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="70" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="G69" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A70" s="1" t="s">
         <v>74</v>
       </c>
@@ -2867,7 +3092,7 @@
         <v>75</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>145</v>
+        <v>283</v>
       </c>
       <c r="E70" s="1" t="s">
         <v>145</v>
@@ -2875,8 +3100,11 @@
       <c r="F70" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="71" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="G70" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A71" s="1" t="s">
         <v>74</v>
       </c>
@@ -2887,7 +3115,7 @@
         <v>77</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>145</v>
+        <v>283</v>
       </c>
       <c r="E71" s="1" t="s">
         <v>145</v>
@@ -2895,8 +3123,11 @@
       <c r="F71" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="72" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="G71" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A72" s="3" t="s">
         <v>74</v>
       </c>
@@ -2906,17 +3137,18 @@
       <c r="C72" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="D72" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="E72" s="3"/>
+      <c r="D72" s="3"/>
+      <c r="E72" s="3" t="s">
+        <v>145</v>
+      </c>
       <c r="F72" s="3"/>
       <c r="G72" s="3"/>
       <c r="H72" s="3"/>
       <c r="I72" s="3"/>
       <c r="J72" s="3"/>
-    </row>
-    <row r="73" spans="1:10" ht="345.6" x14ac:dyDescent="0.3">
+      <c r="K72" s="3"/>
+    </row>
+    <row r="73" spans="1:11" ht="345.6" x14ac:dyDescent="0.3">
       <c r="A73" s="1" t="s">
         <v>79</v>
       </c>
@@ -2927,16 +3159,19 @@
         <v>81</v>
       </c>
       <c r="D73" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="E73" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="E73" s="1" t="s">
+      <c r="F73" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="F73" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="74" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="G73" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
         <v>79</v>
       </c>
@@ -2944,7 +3179,7 @@
         <v>203</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>232</v>
+        <v>283</v>
       </c>
       <c r="E74" s="1" t="s">
         <v>232</v>
@@ -2953,16 +3188,19 @@
         <v>232</v>
       </c>
       <c r="G74" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H74" s="1" t="s">
         <v>248</v>
-      </c>
-      <c r="H74" s="1" t="s">
-        <v>237</v>
       </c>
       <c r="I74" s="1" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="75" spans="1:10" ht="374.4" x14ac:dyDescent="0.3">
+      <c r="J74" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" ht="374.4" x14ac:dyDescent="0.3">
       <c r="A75" s="1" t="s">
         <v>79</v>
       </c>
@@ -2973,16 +3211,19 @@
         <v>83</v>
       </c>
       <c r="D75" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="E75" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="E75" s="1" t="s">
+      <c r="F75" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="F75" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="76" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="G75" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A76" s="1" t="s">
         <v>79</v>
       </c>
@@ -2990,7 +3231,7 @@
         <v>204</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>232</v>
+        <v>283</v>
       </c>
       <c r="E76" s="1" t="s">
         <v>232</v>
@@ -2999,7 +3240,7 @@
         <v>232</v>
       </c>
       <c r="G76" s="1" t="s">
-        <v>249</v>
+        <v>232</v>
       </c>
       <c r="H76" s="1" t="s">
         <v>249</v>
@@ -3007,8 +3248,11 @@
       <c r="I76" s="1" t="s">
         <v>249</v>
       </c>
-    </row>
-    <row r="77" spans="1:10" ht="273.60000000000002" x14ac:dyDescent="0.3">
+      <c r="J76" s="1" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" ht="273.60000000000002" x14ac:dyDescent="0.3">
       <c r="A77" s="1" t="s">
         <v>79</v>
       </c>
@@ -3019,16 +3263,19 @@
         <v>84</v>
       </c>
       <c r="D77" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="E77" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="E77" s="1" t="s">
+      <c r="F77" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="F77" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="78" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G77" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A78" s="1" t="s">
         <v>85</v>
       </c>
@@ -3039,16 +3286,19 @@
         <v>89</v>
       </c>
       <c r="D78" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="E78" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="E78" s="1" t="s">
+      <c r="F78" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="F78" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="79" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="G78" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A79" s="1" t="s">
         <v>85</v>
       </c>
@@ -3056,7 +3306,7 @@
         <v>205</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>232</v>
+        <v>283</v>
       </c>
       <c r="E79" s="1" t="s">
         <v>232</v>
@@ -3065,16 +3315,19 @@
         <v>232</v>
       </c>
       <c r="G79" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H79" s="1" t="s">
         <v>248</v>
-      </c>
-      <c r="H79" s="1" t="s">
-        <v>237</v>
       </c>
       <c r="I79" s="1" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="80" spans="1:10" ht="72" x14ac:dyDescent="0.3">
+      <c r="J79" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" ht="72" x14ac:dyDescent="0.3">
       <c r="A80" s="1" t="s">
         <v>85</v>
       </c>
@@ -3085,16 +3338,19 @@
         <v>91</v>
       </c>
       <c r="D80" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="E80" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="E80" s="1" t="s">
+      <c r="F80" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="F80" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="81" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="G80" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A81" s="1" t="s">
         <v>85</v>
       </c>
@@ -3105,7 +3361,7 @@
         <v>92</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>232</v>
+        <v>283</v>
       </c>
       <c r="E81" s="1" t="s">
         <v>232</v>
@@ -3114,16 +3370,19 @@
         <v>232</v>
       </c>
       <c r="G81" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H81" s="1" t="s">
         <v>248</v>
-      </c>
-      <c r="H81" s="1" t="s">
-        <v>237</v>
       </c>
       <c r="I81" s="1" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="82" spans="1:10" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="J81" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A82" s="1" t="s">
         <v>85</v>
       </c>
@@ -3134,16 +3393,19 @@
         <v>93</v>
       </c>
       <c r="D82" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="E82" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="E82" s="1" t="s">
+      <c r="F82" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="F82" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="83" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="G82" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A83" s="1" t="s">
         <v>85</v>
       </c>
@@ -3153,17 +3415,20 @@
       <c r="C83" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="D83" s="1" t="s">
+      <c r="D83" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="E83" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="E83" s="1" t="s">
+      <c r="F83" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="F83" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="84" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="G83" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A84" s="1" t="s">
         <v>85</v>
       </c>
@@ -3171,8 +3436,8 @@
         <v>206</v>
       </c>
       <c r="C84" s="2"/>
-      <c r="D84" s="1" t="s">
-        <v>232</v>
+      <c r="D84" s="2" t="s">
+        <v>283</v>
       </c>
       <c r="E84" s="1" t="s">
         <v>232</v>
@@ -3181,16 +3446,19 @@
         <v>232</v>
       </c>
       <c r="G84" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H84" s="1" t="s">
         <v>248</v>
-      </c>
-      <c r="H84" s="1" t="s">
-        <v>237</v>
       </c>
       <c r="I84" s="1" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="85" spans="1:10" ht="72" x14ac:dyDescent="0.3">
+      <c r="J84" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11" ht="72" x14ac:dyDescent="0.3">
       <c r="A85" s="1" t="s">
         <v>97</v>
       </c>
@@ -3201,16 +3469,19 @@
         <v>98</v>
       </c>
       <c r="D85" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="E85" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="E85" s="1" t="s">
+      <c r="F85" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="F85" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="86" spans="1:10" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="G85" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A86" s="1" t="s">
         <v>97</v>
       </c>
@@ -3220,8 +3491,8 @@
       <c r="C86" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="D86" s="1" t="s">
-        <v>232</v>
+      <c r="D86" s="2" t="s">
+        <v>283</v>
       </c>
       <c r="E86" s="1" t="s">
         <v>232</v>
@@ -3230,16 +3501,19 @@
         <v>232</v>
       </c>
       <c r="G86" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H86" s="1" t="s">
         <v>250</v>
-      </c>
-      <c r="H86" s="1" t="s">
-        <v>237</v>
       </c>
       <c r="I86" s="1" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="87" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="J86" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A87" s="1" t="s">
         <v>97</v>
       </c>
@@ -3250,16 +3524,19 @@
         <v>104</v>
       </c>
       <c r="D87" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="E87" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="E87" s="1" t="s">
+      <c r="F87" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="F87" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="88" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="G87" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="88" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A88" s="1" t="s">
         <v>97</v>
       </c>
@@ -3270,19 +3547,22 @@
         <v>105</v>
       </c>
       <c r="D88" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="E88" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="E88" s="1" t="s">
+      <c r="F88" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="F88" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="J88" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="89" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="G88" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="K88" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="89" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A89" s="1" t="s">
         <v>97</v>
       </c>
@@ -3293,19 +3573,22 @@
         <v>106</v>
       </c>
       <c r="D89" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="E89" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="E89" s="1" t="s">
+      <c r="F89" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="F89" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="J89" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="90" spans="1:10" ht="72" x14ac:dyDescent="0.3">
+      <c r="G89" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="K89" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="90" spans="1:11" ht="72" x14ac:dyDescent="0.3">
       <c r="A90" s="1" t="s">
         <v>108</v>
       </c>
@@ -3316,7 +3599,7 @@
         <v>110</v>
       </c>
       <c r="D90" s="1" t="s">
-        <v>232</v>
+        <v>283</v>
       </c>
       <c r="E90" s="1" t="s">
         <v>232</v>
@@ -3325,16 +3608,19 @@
         <v>232</v>
       </c>
       <c r="G90" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H90" s="1" t="s">
         <v>251</v>
-      </c>
-      <c r="H90" s="1" t="s">
-        <v>237</v>
       </c>
       <c r="I90" s="1" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="91" spans="1:10" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="J90" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="91" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A91" s="1" t="s">
         <v>108</v>
       </c>
@@ -3345,7 +3631,7 @@
         <v>112</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>232</v>
+        <v>283</v>
       </c>
       <c r="E91" s="1" t="s">
         <v>232</v>
@@ -3354,16 +3640,19 @@
         <v>232</v>
       </c>
       <c r="G91" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H91" s="1" t="s">
         <v>251</v>
-      </c>
-      <c r="H91" s="1" t="s">
-        <v>237</v>
       </c>
       <c r="I91" s="1" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="92" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="J91" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="92" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A92" s="1" t="s">
         <v>108</v>
       </c>
@@ -3374,7 +3663,7 @@
         <v>117</v>
       </c>
       <c r="D92" s="1" t="s">
-        <v>232</v>
+        <v>283</v>
       </c>
       <c r="E92" s="1" t="s">
         <v>232</v>
@@ -3383,19 +3672,22 @@
         <v>232</v>
       </c>
       <c r="G92" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H92" s="1" t="s">
         <v>251</v>
-      </c>
-      <c r="H92" s="1" t="s">
-        <v>237</v>
       </c>
       <c r="I92" s="1" t="s">
         <v>237</v>
       </c>
       <c r="J92" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="93" spans="1:10" ht="72" x14ac:dyDescent="0.3">
+        <v>237</v>
+      </c>
+      <c r="K92" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="93" spans="1:11" ht="72" x14ac:dyDescent="0.3">
       <c r="A93" s="1" t="s">
         <v>108</v>
       </c>
@@ -3406,7 +3698,7 @@
         <v>118</v>
       </c>
       <c r="D93" s="1" t="s">
-        <v>232</v>
+        <v>283</v>
       </c>
       <c r="E93" s="1" t="s">
         <v>232</v>
@@ -3415,19 +3707,22 @@
         <v>232</v>
       </c>
       <c r="G93" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H93" s="1" t="s">
         <v>251</v>
-      </c>
-      <c r="H93" s="1" t="s">
-        <v>237</v>
       </c>
       <c r="I93" s="1" t="s">
         <v>237</v>
       </c>
       <c r="J93" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="94" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+        <v>237</v>
+      </c>
+      <c r="K93" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="94" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A94" s="1" t="s">
         <v>108</v>
       </c>
@@ -3438,16 +3733,19 @@
         <v>120</v>
       </c>
       <c r="D94" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="E94" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="E94" s="1" t="s">
+      <c r="F94" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="F94" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="95" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G94" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="95" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A95" s="1" t="s">
         <v>108</v>
       </c>
@@ -3458,7 +3756,7 @@
         <v>119</v>
       </c>
       <c r="D95" s="1" t="s">
-        <v>232</v>
+        <v>283</v>
       </c>
       <c r="E95" s="1" t="s">
         <v>232</v>
@@ -3467,19 +3765,22 @@
         <v>232</v>
       </c>
       <c r="G95" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H95" s="1" t="s">
         <v>252</v>
       </c>
-      <c r="H95" s="1" t="s">
+      <c r="I95" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="I95" s="1" t="s">
+      <c r="J95" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="J95" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="96" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="K95" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="96" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A96" s="1" t="s">
         <v>108</v>
       </c>
@@ -3490,7 +3791,7 @@
         <v>121</v>
       </c>
       <c r="D96" s="1" t="s">
-        <v>232</v>
+        <v>283</v>
       </c>
       <c r="E96" s="1" t="s">
         <v>232</v>
@@ -3499,19 +3800,22 @@
         <v>232</v>
       </c>
       <c r="G96" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H96" s="1" t="s">
         <v>252</v>
       </c>
-      <c r="H96" s="1" t="s">
+      <c r="I96" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="I96" s="1" t="s">
+      <c r="J96" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="J96" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="97" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="K96" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="97" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A97" s="1" t="s">
         <v>108</v>
       </c>
@@ -3522,19 +3826,22 @@
         <v>122</v>
       </c>
       <c r="D97" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="E97" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="E97" s="1" t="s">
+      <c r="F97" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="F97" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="J97" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="98" spans="1:10" ht="72" x14ac:dyDescent="0.3">
+      <c r="G97" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="K97" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="98" spans="1:11" ht="72" x14ac:dyDescent="0.3">
       <c r="A98" s="1" t="s">
         <v>108</v>
       </c>
@@ -3545,7 +3852,7 @@
         <v>123</v>
       </c>
       <c r="D98" s="1" t="s">
-        <v>145</v>
+        <v>281</v>
       </c>
       <c r="E98" s="1" t="s">
         <v>145</v>
@@ -3553,8 +3860,11 @@
       <c r="F98" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="99" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="G98" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="99" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A99" s="1" t="s">
         <v>108</v>
       </c>
@@ -3565,7 +3875,7 @@
         <v>209</v>
       </c>
       <c r="D99" s="1" t="s">
-        <v>232</v>
+        <v>281</v>
       </c>
       <c r="E99" s="1" t="s">
         <v>232</v>
@@ -3574,16 +3884,19 @@
         <v>232</v>
       </c>
       <c r="G99" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H99" s="1" t="s">
         <v>255</v>
-      </c>
-      <c r="H99" s="1" t="s">
-        <v>256</v>
       </c>
       <c r="I99" s="1" t="s">
         <v>256</v>
       </c>
-    </row>
-    <row r="100" spans="1:10" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="J99" s="1" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="100" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A100" s="1" t="s">
         <v>108</v>
       </c>
@@ -3594,7 +3907,7 @@
         <v>124</v>
       </c>
       <c r="D100" s="1" t="s">
-        <v>145</v>
+        <v>281</v>
       </c>
       <c r="E100" s="1" t="s">
         <v>145</v>
@@ -3602,8 +3915,11 @@
       <c r="F100" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="101" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="G100" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="101" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A101" s="1" t="s">
         <v>108</v>
       </c>
@@ -3611,7 +3927,7 @@
         <v>211</v>
       </c>
       <c r="D101" s="1" t="s">
-        <v>232</v>
+        <v>281</v>
       </c>
       <c r="E101" s="1" t="s">
         <v>232</v>
@@ -3620,16 +3936,19 @@
         <v>232</v>
       </c>
       <c r="G101" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H101" s="1" t="s">
         <v>257</v>
-      </c>
-      <c r="H101" s="1" t="s">
-        <v>258</v>
       </c>
       <c r="I101" s="1" t="s">
         <v>258</v>
       </c>
-    </row>
-    <row r="102" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="J101" s="1" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="102" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A102" s="1" t="s">
         <v>108</v>
       </c>
@@ -3640,7 +3959,7 @@
         <v>125</v>
       </c>
       <c r="D102" s="1" t="s">
-        <v>145</v>
+        <v>281</v>
       </c>
       <c r="E102" s="1" t="s">
         <v>145</v>
@@ -3648,8 +3967,11 @@
       <c r="F102" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="103" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="G102" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="103" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A103" s="1" t="s">
         <v>108</v>
       </c>
@@ -3657,7 +3979,7 @@
         <v>212</v>
       </c>
       <c r="D103" s="1" t="s">
-        <v>232</v>
+        <v>281</v>
       </c>
       <c r="E103" s="1" t="s">
         <v>232</v>
@@ -3666,16 +3988,19 @@
         <v>232</v>
       </c>
       <c r="G103" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H103" s="1" t="s">
         <v>259</v>
-      </c>
-      <c r="H103" s="1" t="s">
-        <v>260</v>
       </c>
       <c r="I103" s="1" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="104" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="J103" s="1" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="104" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A104" s="1" t="s">
         <v>126</v>
       </c>
@@ -3686,7 +4011,7 @@
         <v>128</v>
       </c>
       <c r="D104" s="1" t="s">
-        <v>145</v>
+        <v>281</v>
       </c>
       <c r="E104" s="1" t="s">
         <v>145</v>
@@ -3694,8 +4019,11 @@
       <c r="F104" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="105" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="G104" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="105" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A105" s="1" t="s">
         <v>126</v>
       </c>
@@ -3706,7 +4034,7 @@
         <v>152</v>
       </c>
       <c r="D105" s="1" t="s">
-        <v>145</v>
+        <v>281</v>
       </c>
       <c r="E105" s="1" t="s">
         <v>145</v>
@@ -3717,8 +4045,11 @@
       <c r="G105" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="106" spans="1:10" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="H105" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="106" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A106" s="1" t="s">
         <v>126</v>
       </c>
@@ -3729,7 +4060,7 @@
         <v>135</v>
       </c>
       <c r="D106" s="1" t="s">
-        <v>261</v>
+        <v>281</v>
       </c>
       <c r="E106" s="1" t="s">
         <v>261</v>
@@ -3738,16 +4069,19 @@
         <v>261</v>
       </c>
       <c r="G106" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="H106" s="1" t="s">
         <v>262</v>
-      </c>
-      <c r="H106" s="1" t="s">
-        <v>263</v>
       </c>
       <c r="I106" s="1" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="107" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="J106" s="1" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="107" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A107" s="1" t="s">
         <v>126</v>
       </c>
@@ -3758,7 +4092,7 @@
         <v>136</v>
       </c>
       <c r="D107" s="1" t="s">
-        <v>264</v>
+        <v>281</v>
       </c>
       <c r="E107" s="1" t="s">
         <v>264</v>
@@ -3766,8 +4100,11 @@
       <c r="F107" s="1" t="s">
         <v>264</v>
       </c>
-    </row>
-    <row r="108" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="G107" s="1" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="108" spans="1:11" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A108" s="1" t="s">
         <v>126</v>
       </c>
@@ -3775,7 +4112,7 @@
         <v>214</v>
       </c>
       <c r="D108" s="1" t="s">
-        <v>232</v>
+        <v>281</v>
       </c>
       <c r="E108" s="1" t="s">
         <v>232</v>
@@ -3784,16 +4121,19 @@
         <v>232</v>
       </c>
       <c r="G108" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H108" s="1" t="s">
         <v>265</v>
-      </c>
-      <c r="H108" s="1" t="s">
-        <v>266</v>
       </c>
       <c r="I108" s="1" t="s">
         <v>266</v>
       </c>
-    </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J108" s="1" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="109" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A109" s="1" t="s">
         <v>126</v>
       </c>
@@ -3801,7 +4141,7 @@
         <v>137</v>
       </c>
       <c r="D109" s="1" t="s">
-        <v>145</v>
+        <v>281</v>
       </c>
       <c r="E109" s="1" t="s">
         <v>145</v>
@@ -3809,8 +4149,11 @@
       <c r="F109" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="110" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G109" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="110" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A110" s="1" t="s">
         <v>126</v>
       </c>
@@ -3818,7 +4161,7 @@
         <v>215</v>
       </c>
       <c r="D110" s="1" t="s">
-        <v>232</v>
+        <v>281</v>
       </c>
       <c r="E110" s="1" t="s">
         <v>232</v>
@@ -3827,16 +4170,19 @@
         <v>232</v>
       </c>
       <c r="G110" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H110" s="1" t="s">
         <v>267</v>
       </c>
-      <c r="H110" s="1" t="s">
-        <v>145</v>
-      </c>
       <c r="I110" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J110" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="111" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A111" s="1" t="s">
         <v>126</v>
       </c>
@@ -3847,7 +4193,7 @@
         <v>216</v>
       </c>
       <c r="D111" s="1" t="s">
-        <v>145</v>
+        <v>281</v>
       </c>
       <c r="E111" s="1" t="s">
         <v>145</v>
@@ -3855,8 +4201,11 @@
       <c r="F111" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="G111" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="112" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A112" s="1" t="s">
         <v>126</v>
       </c>
@@ -3867,7 +4216,7 @@
         <v>217</v>
       </c>
       <c r="D112" s="1" t="s">
-        <v>145</v>
+        <v>281</v>
       </c>
       <c r="E112" s="1" t="s">
         <v>145</v>
@@ -3875,8 +4224,11 @@
       <c r="F112" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="113" spans="1:9" ht="72" x14ac:dyDescent="0.3">
+      <c r="G112" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="113" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A113" s="1" t="s">
         <v>126</v>
       </c>
@@ -3887,7 +4239,7 @@
         <v>141</v>
       </c>
       <c r="D113" s="1" t="s">
-        <v>232</v>
+        <v>281</v>
       </c>
       <c r="E113" s="1" t="s">
         <v>232</v>
@@ -3896,16 +4248,19 @@
         <v>232</v>
       </c>
       <c r="G113" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H113" s="1" t="s">
         <v>268</v>
-      </c>
-      <c r="H113" s="1" t="s">
-        <v>269</v>
       </c>
       <c r="I113" s="1" t="s">
         <v>269</v>
       </c>
-    </row>
-    <row r="114" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="J113" s="1" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="114" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A114" s="1" t="s">
         <v>126</v>
       </c>
@@ -3916,7 +4271,7 @@
         <v>143</v>
       </c>
       <c r="D114" s="1" t="s">
-        <v>270</v>
+        <v>281</v>
       </c>
       <c r="E114" s="1" t="s">
         <v>270</v>
@@ -3924,8 +4279,11 @@
       <c r="F114" s="1" t="s">
         <v>270</v>
       </c>
-    </row>
-    <row r="115" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="G114" s="1" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="115" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A115" s="1" t="s">
         <v>126</v>
       </c>
@@ -3933,12 +4291,15 @@
         <v>144</v>
       </c>
       <c r="D115" s="1" t="s">
-        <v>270</v>
+        <v>281</v>
       </c>
       <c r="E115" s="1" t="s">
         <v>270</v>
       </c>
       <c r="F115" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="G115" s="1" t="s">
         <v>270</v>
       </c>
     </row>

</xml_diff>

<commit_message>
framework updates for AIVisualize
</commit_message>
<xml_diff>
--- a/_context/AEO_TOOL_MAPPING_V1.xlsx
+++ b/_context/AEO_TOOL_MAPPING_V1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MyApps\aeo-audit-tool-v3\_context\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{943D01EF-253F-48CD-9F66-0DA441123AFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD92C3DB-345C-41CC-A5B5-CAF37567C3E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6073F0D8-4F6F-4048-AC8C-2714F136D76E}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1065" uniqueCount="329">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1058" uniqueCount="328">
   <si>
     <t>AISocialize</t>
   </si>
@@ -489,9 +489,6 @@
     <t>X</t>
   </si>
   <si>
-    <t>ai-context.md basic file availability</t>
-  </si>
-  <si>
     <t>README.md Updates</t>
   </si>
   <si>
@@ -1005,9 +1002,6 @@
     <t>EXEC(Yes/no)-DIY(details/link)</t>
   </si>
   <si>
-    <t>DI(mention as upgrade from HasFAQSchema)</t>
-  </si>
-  <si>
     <t>Answer corrections (Per page)</t>
   </si>
   <si>
@@ -1039,6 +1033,9 @@
   </si>
   <si>
     <t>Upgrade from Headerscheck</t>
+  </si>
+  <si>
+    <t>DIY(mention as upgrade from HasFAQSchema)</t>
   </si>
 </sst>
 </file>
@@ -1187,10 +1184,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FD337438-C06E-4F50-BBED-8980A160B1E2}" name="Table1" displayName="Table1" ref="A1:N115" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
-  <autoFilter ref="A1:N115" xr:uid="{FD337438-C06E-4F50-BBED-8980A160B1E2}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N115">
-    <sortCondition ref="B1:B115"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FD337438-C06E-4F50-BBED-8980A160B1E2}" name="Table1" displayName="Table1" ref="A1:N114" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
+  <autoFilter ref="A1:N114" xr:uid="{FD337438-C06E-4F50-BBED-8980A160B1E2}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N114">
+    <sortCondition ref="A1:A114"/>
   </sortState>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{EA71DEFB-ED09-4AF2-B003-CFBC5B42A87C}" name="no." dataDxfId="20"/>
@@ -1545,7 +1542,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55A4A3A0-5979-416B-A6BF-400E246F3969}">
-  <dimension ref="A1:N115"/>
+  <dimension ref="A1:N114"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.44140625" style="1" bestFit="1" customWidth="1"/>
@@ -1562,10 +1559,10 @@
   <sheetData>
     <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>304</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>305</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -1574,31 +1571,31 @@
         <v>51</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>228</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>229</v>
       </c>
       <c r="N1" s="1" t="s">
         <v>0</v>
@@ -1612,16 +1609,16 @@
         <v>22</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>144</v>
@@ -1641,10 +1638,10 @@
         <v>36</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="H3" s="1" t="s">
         <v>144</v>
@@ -1667,22 +1664,22 @@
         <v>37</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="K4" s="1" t="s">
         <v>144</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="129.6" x14ac:dyDescent="0.3">
@@ -1699,31 +1696,31 @@
         <v>102</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F5" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>306</v>
       </c>
-      <c r="G5" s="2" t="s">
-        <v>307</v>
-      </c>
       <c r="H5" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="72" x14ac:dyDescent="0.3">
@@ -1740,16 +1737,16 @@
         <v>97</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="H6" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="I6" s="1" t="s">
         <v>272</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>273</v>
       </c>
       <c r="J6" s="1" t="s">
         <v>144</v>
@@ -1769,16 +1766,16 @@
         <v>103</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="H7" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="I7" s="1" t="s">
         <v>272</v>
-      </c>
-      <c r="I7" s="1" t="s">
-        <v>273</v>
       </c>
       <c r="J7" s="1" t="s">
         <v>144</v>
@@ -1798,16 +1795,16 @@
         <v>104</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="H8" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="I8" s="1" t="s">
         <v>272</v>
-      </c>
-      <c r="I8" s="1" t="s">
-        <v>273</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>144</v>
@@ -1830,16 +1827,16 @@
         <v>105</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="H9" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="I9" s="1" t="s">
         <v>272</v>
-      </c>
-      <c r="I9" s="1" t="s">
-        <v>273</v>
       </c>
       <c r="J9" s="1" t="s">
         <v>144</v>
@@ -1862,16 +1859,16 @@
         <v>53</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="H10" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="I10" s="1" t="s">
         <v>268</v>
-      </c>
-      <c r="I10" s="1" t="s">
-        <v>269</v>
       </c>
       <c r="J10" s="1" t="s">
         <v>144</v>
@@ -1891,10 +1888,10 @@
         <v>52</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="H11" s="1" t="s">
         <v>144</v>
@@ -1914,37 +1911,37 @@
         <v>18</v>
       </c>
       <c r="C12" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="K12" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="L12" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="D12" s="1" t="s">
-        <v>234</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>293</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="H12" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="I12" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="J12" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="K12" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="L12" s="1" t="s">
-        <v>233</v>
-      </c>
       <c r="M12" s="1" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="13" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -1955,16 +1952,16 @@
         <v>18</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="I13" s="1" t="s">
         <v>144</v>
@@ -1984,10 +1981,10 @@
         <v>42</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>303</v>
+        <v>281</v>
       </c>
       <c r="H14" s="1" t="s">
         <v>144</v>
@@ -2010,10 +2007,10 @@
         <v>43</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="H15" s="1" t="s">
         <v>144</v>
@@ -2036,10 +2033,10 @@
         <v>45</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="H16" s="1" t="s">
         <v>144</v>
@@ -2051,219 +2048,231 @@
         <v>144</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>145</v>
+        <v>44</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F17" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A18" s="1">
+        <v>18</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="L18" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="M18" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A19" s="1">
+        <v>19</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>282</v>
       </c>
-      <c r="H17" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="I17" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="J17" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="1">
-        <v>17</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>310</v>
-      </c>
-      <c r="H18" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="I18" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="J18" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A19" s="1">
-        <v>18</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>293</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>298</v>
-      </c>
       <c r="H19" s="1" t="s">
-        <v>230</v>
+        <v>144</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>230</v>
+        <v>144</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="K19" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="L19" s="1" t="s">
-        <v>233</v>
-      </c>
-      <c r="M19" s="1" t="s">
-        <v>233</v>
+        <v>144</v>
+      </c>
+      <c r="N19" s="1" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="20" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>68</v>
+        <v>26</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>69</v>
+        <v>7</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>283</v>
+        <v>310</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>144</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>144</v>
+        <v>229</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>144</v>
+        <v>229</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="N20" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="21" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+        <v>229</v>
+      </c>
+      <c r="K20" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="L20" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="M20" s="1" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>26</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>311</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>144</v>
+        <v>289</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="I21" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="J21" s="1" t="s">
-        <v>230</v>
+        <v>144</v>
       </c>
       <c r="K21" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="L21" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="M21" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F22" s="1" t="s">
         <v>290</v>
       </c>
+      <c r="G22" s="1" t="s">
+        <v>144</v>
+      </c>
       <c r="H22" s="1" t="s">
-        <v>144</v>
+        <v>229</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="J22" s="1" t="s">
+        <v>229</v>
       </c>
       <c r="K22" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="L22" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="M22" s="1" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="23" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>27</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="G23" s="1" t="s">
         <v>144</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="K23" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="L23" s="1" t="s">
         <v>144</v>
@@ -2274,34 +2283,34 @@
     </row>
     <row r="24" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>27</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="G24" s="1" t="s">
         <v>144</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="L24" s="1" t="s">
         <v>144</v>
@@ -2310,106 +2319,97 @@
         <v>144</v>
       </c>
     </row>
-    <row r="25" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>10</v>
+        <v>222</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>238</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="G25" s="1" t="s">
         <v>144</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>230</v>
+        <v>144</v>
       </c>
       <c r="L25" s="1" t="s">
-        <v>144</v>
+        <v>232</v>
       </c>
       <c r="M25" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="26" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+        <v>232</v>
+      </c>
+      <c r="N25" s="1" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>23</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>239</v>
+        <v>195</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>295</v>
-      </c>
-      <c r="G26" s="1" t="s">
-        <v>144</v>
+        <v>282</v>
       </c>
       <c r="H26" s="1" t="s">
         <v>230</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>230</v>
+        <v>144</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="K26" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="L26" s="1" t="s">
-        <v>233</v>
-      </c>
-      <c r="M26" s="1" t="s">
-        <v>233</v>
+        <v>144</v>
       </c>
       <c r="N26" s="1" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="27" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>23</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>196</v>
+        <v>41</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>231</v>
+        <v>144</v>
       </c>
       <c r="I27" s="1" t="s">
         <v>144</v>
@@ -2423,16 +2423,16 @@
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>23</v>
+        <v>50</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>41</v>
+        <v>196</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>282</v>
@@ -2446,13 +2446,10 @@
       <c r="J28" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="N28" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
+    </row>
+    <row r="29" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>50</v>
@@ -2461,10 +2458,10 @@
         <v>197</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="H29" s="1" t="s">
         <v>144</v>
@@ -2476,73 +2473,73 @@
         <v>144</v>
       </c>
     </row>
-    <row r="30" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="C30" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="H30" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="I30" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="J30" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="K30" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="L30" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="M30" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A31" s="1">
+        <v>31</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C31" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="E30" s="1" t="s">
-        <v>279</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>283</v>
-      </c>
-      <c r="H30" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="I30" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="J30" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="31" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A31" s="1">
-        <v>30</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>58</v>
-      </c>
       <c r="E31" s="1" t="s">
-        <v>279</v>
-      </c>
-      <c r="G31" s="1" t="s">
-        <v>300</v>
+        <v>278</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>282</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>230</v>
+        <v>144</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>230</v>
+        <v>144</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="K31" s="1" t="s">
-        <v>240</v>
-      </c>
-      <c r="L31" s="1" t="s">
-        <v>233</v>
-      </c>
-      <c r="M31" s="1" t="s">
-        <v>233</v>
+        <v>144</v>
       </c>
     </row>
     <row r="32" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>73</v>
@@ -2550,11 +2547,14 @@
       <c r="C32" s="1" t="s">
         <v>199</v>
       </c>
+      <c r="D32" s="1" t="s">
+        <v>74</v>
+      </c>
       <c r="E32" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="H32" s="1" t="s">
         <v>144</v>
@@ -2568,263 +2568,272 @@
     </row>
     <row r="33" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>73</v>
       </c>
       <c r="C33" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="H33" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="I33" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="J33" s="1" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A34" s="1">
+        <v>34</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="D34" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="D33" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="E33" s="1" t="s">
-        <v>279</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>283</v>
-      </c>
-      <c r="H33" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="I33" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="J33" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="34" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A34" s="1">
-        <v>33</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>279</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>283</v>
-      </c>
-      <c r="H34" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="I34" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="J34" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="35" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="E34" s="3"/>
+      <c r="F34" s="3"/>
+      <c r="G34" s="3"/>
+      <c r="H34" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="I34" s="3"/>
+      <c r="J34" s="3"/>
+      <c r="K34" s="3"/>
+      <c r="L34" s="3"/>
+      <c r="M34" s="3"/>
+      <c r="N34" s="3"/>
+    </row>
+    <row r="35" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A35" s="1">
-        <v>34</v>
-      </c>
-      <c r="B35" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="C35" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="D35" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="E35" s="3"/>
-      <c r="F35" s="3"/>
-      <c r="G35" s="3"/>
-      <c r="H35" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="I35" s="3"/>
-      <c r="J35" s="3"/>
-      <c r="K35" s="3"/>
-      <c r="L35" s="3"/>
-      <c r="M35" s="3"/>
-      <c r="N35" s="3"/>
+        <v>35</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>311</v>
+      </c>
+      <c r="H35" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="I35" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="J35" s="1" t="s">
+        <v>144</v>
+      </c>
     </row>
     <row r="36" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A36" s="1">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>70</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>71</v>
+        <v>241</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>72</v>
+        <v>242</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>312</v>
+        <v>282</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>231</v>
-      </c>
-      <c r="I36" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="J36" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="37" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A37" s="1">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>242</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>243</v>
+        <v>64</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>279</v>
-      </c>
-      <c r="F37" s="1" t="s">
-        <v>283</v>
+        <v>278</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>300</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>144</v>
+        <v>229</v>
+      </c>
+      <c r="I37" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="J37" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="K37" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="L37" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="M37" s="1" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="38" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A38" s="1">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>60</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="K38" s="1" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="L38" s="1" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="M38" s="1" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="39" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A39" s="1">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>60</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>279</v>
-      </c>
-      <c r="G39" s="1" t="s">
-        <v>301</v>
+        <v>278</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>283</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>230</v>
+        <v>144</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>230</v>
+        <v>144</v>
       </c>
       <c r="J39" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="K39" s="1" t="s">
-        <v>241</v>
-      </c>
-      <c r="L39" s="1" t="s">
-        <v>233</v>
-      </c>
-      <c r="M39" s="1" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="40" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A40" s="1">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>60</v>
+        <v>17</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>63</v>
+        <v>34</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>279</v>
-      </c>
-      <c r="F40" s="1" t="s">
-        <v>284</v>
+        <v>276</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>291</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>144</v>
+        <v>229</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>144</v>
+        <v>229</v>
       </c>
       <c r="J40" s="1" t="s">
-        <v>144</v>
+        <v>229</v>
+      </c>
+      <c r="K40" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="L40" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="M40" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="N40" s="1" t="s">
+        <v>229</v>
       </c>
     </row>
     <row r="41" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A41" s="1">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I41" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="J41" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="K41" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="L41" s="1" t="s">
         <v>144</v>
@@ -2833,62 +2842,53 @@
         <v>144</v>
       </c>
       <c r="N41" s="1" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="42" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A42" s="1">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="G42" s="1" t="s">
-        <v>292</v>
+        <v>276</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>281</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>230</v>
+        <v>144</v>
       </c>
       <c r="I42" s="1" t="s">
-        <v>230</v>
+        <v>144</v>
       </c>
       <c r="J42" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="K42" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="L42" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="M42" s="1" t="s">
         <v>144</v>
       </c>
       <c r="N42" s="1" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A43" s="1">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>282</v>
+        <v>309</v>
       </c>
       <c r="H43" s="1" t="s">
         <v>144</v>
@@ -2903,21 +2903,21 @@
         <v>144</v>
       </c>
     </row>
-    <row r="44" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A44" s="1">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B44" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>33</v>
+        <v>191</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>310</v>
+        <v>282</v>
       </c>
       <c r="H44" s="1" t="s">
         <v>144</v>
@@ -2934,62 +2934,50 @@
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A45" s="1">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>192</v>
+        <v>56</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="F45" s="1" t="s">
-        <v>283</v>
-      </c>
-      <c r="H45" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="I45" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="J45" s="1" t="s">
-        <v>144</v>
+        <v>280</v>
       </c>
       <c r="N45" s="1" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A46" s="1">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="N46" s="1" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="47" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A47" s="1">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="N47" s="1" t="s">
         <v>144</v>
@@ -2997,88 +2985,103 @@
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A48" s="1">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>17</v>
+        <v>147</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>66</v>
+        <v>146</v>
       </c>
       <c r="E48" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="F48" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="N48" s="1" t="s">
+      <c r="H48" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="I48" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="J48" s="1" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A49" s="1">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B49" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="F49" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="H49" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="I49" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="J49" s="1" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A50" s="1">
+        <v>50</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="F50" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="H50" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="I50" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="J50" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="N50" s="1" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A51" s="1">
+        <v>51</v>
+      </c>
+      <c r="B51" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="C49" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="E49" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="F49" s="1" t="s">
-        <v>282</v>
-      </c>
-      <c r="H49" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="I49" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="J49" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A50" s="1">
-        <v>49</v>
-      </c>
-      <c r="B50" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="C50" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="E50" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="F50" s="1" t="s">
-        <v>282</v>
-      </c>
-      <c r="H50" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="I50" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="J50" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="51" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A51" s="1">
-        <v>50</v>
-      </c>
-      <c r="B51" s="1" t="s">
-        <v>178</v>
-      </c>
       <c r="C51" s="1" t="s">
-        <v>179</v>
+        <v>149</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>310</v>
+        <v>292</v>
+      </c>
+      <c r="G51" s="1" t="s">
+        <v>297</v>
       </c>
       <c r="H51" s="1" t="s">
         <v>144</v>
@@ -3089,192 +3092,201 @@
       <c r="J51" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="N51" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="52" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="52" spans="1:14" ht="72" x14ac:dyDescent="0.3">
       <c r="A52" s="1">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>149</v>
+        <v>107</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>150</v>
+        <v>108</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>109</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>293</v>
-      </c>
-      <c r="G52" s="1" t="s">
-        <v>298</v>
+        <v>312</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>144</v>
+        <v>229</v>
       </c>
       <c r="I52" s="1" t="s">
-        <v>144</v>
+        <v>229</v>
       </c>
       <c r="J52" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="53" spans="1:14" ht="72" x14ac:dyDescent="0.3">
+        <v>229</v>
+      </c>
+      <c r="K52" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="L52" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="M52" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A53" s="1">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B53" s="1" t="s">
         <v>107</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="H53" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I53" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="J53" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="K53" s="1" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="L53" s="1" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="M53" s="1" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="54" spans="1:14" ht="86.4" x14ac:dyDescent="0.3">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A54" s="1">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B54" s="1" t="s">
         <v>107</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I54" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="J54" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="K54" s="1" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="L54" s="1" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="M54" s="1" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="55" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+        <v>232</v>
+      </c>
+      <c r="N54" s="1" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="55" spans="1:14" ht="72" x14ac:dyDescent="0.3">
       <c r="A55" s="1">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B55" s="1" t="s">
         <v>107</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="H55" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I55" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="J55" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="K55" s="1" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="L55" s="1" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="M55" s="1" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="N55" s="1" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="56" spans="1:14" ht="72" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A56" s="1">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B56" s="1" t="s">
         <v>107</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>113</v>
+        <v>274</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="H56" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I56" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="J56" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="K56" s="1" t="s">
         <v>247</v>
       </c>
       <c r="L56" s="1" t="s">
-        <v>233</v>
+        <v>248</v>
       </c>
       <c r="M56" s="1" t="s">
-        <v>233</v>
+        <v>249</v>
       </c>
       <c r="N56" s="1" t="s">
         <v>144</v>
@@ -3282,7 +3294,7 @@
     </row>
     <row r="57" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A57" s="1">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B57" s="1" t="s">
         <v>107</v>
@@ -3291,118 +3303,112 @@
         <v>275</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I57" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="J57" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="K57" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="L57" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="L57" s="1" t="s">
+      <c r="M57" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="M57" s="1" t="s">
-        <v>250</v>
-      </c>
       <c r="N57" s="1" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="58" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A58" s="1">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B58" s="1" t="s">
         <v>107</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>276</v>
+        <v>205</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>120</v>
+        <v>206</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="H58" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I58" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="J58" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="K58" s="1" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="L58" s="1" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="M58" s="1" t="s">
-        <v>250</v>
-      </c>
-      <c r="N58" s="1" t="s">
-        <v>144</v>
+        <v>251</v>
       </c>
     </row>
     <row r="59" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A59" s="1">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B59" s="1" t="s">
         <v>107</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="D59" s="1" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="H59" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I59" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="J59" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="K59" s="1" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="L59" s="1" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="M59" s="1" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="60" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A60" s="1">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B60" s="1" t="s">
         <v>107</v>
@@ -3411,80 +3417,74 @@
         <v>209</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="H60" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I60" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="J60" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="K60" s="1" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="L60" s="1" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="M60" s="1" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="61" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="61" spans="1:14" ht="72" x14ac:dyDescent="0.3">
       <c r="A61" s="1">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B61" s="1" t="s">
         <v>107</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>210</v>
+        <v>204</v>
+      </c>
+      <c r="D61" s="1" t="s">
+        <v>122</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F61" s="1" t="s">
         <v>313</v>
       </c>
       <c r="H61" s="1" t="s">
-        <v>230</v>
+        <v>144</v>
       </c>
       <c r="I61" s="1" t="s">
-        <v>230</v>
+        <v>144</v>
       </c>
       <c r="J61" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="K61" s="1" t="s">
-        <v>255</v>
-      </c>
-      <c r="L61" s="1" t="s">
-        <v>256</v>
-      </c>
-      <c r="M61" s="1" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="62" spans="1:14" ht="72" x14ac:dyDescent="0.3">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="62" spans="1:14" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A62" s="1">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B62" s="1" t="s">
         <v>107</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F62" s="1" t="s">
         <v>314</v>
@@ -3499,21 +3499,21 @@
         <v>144</v>
       </c>
     </row>
-    <row r="63" spans="1:14" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A63" s="1">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B63" s="1" t="s">
         <v>107</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>208</v>
+        <v>115</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F63" s="1" t="s">
         <v>315</v>
@@ -3528,30 +3528,30 @@
         <v>144</v>
       </c>
     </row>
-    <row r="64" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A64" s="1">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B64" s="1" t="s">
         <v>107</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>115</v>
+        <v>273</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>316</v>
+        <v>282</v>
       </c>
       <c r="H64" s="1" t="s">
-        <v>144</v>
+        <v>271</v>
       </c>
       <c r="I64" s="1" t="s">
-        <v>144</v>
+        <v>272</v>
       </c>
       <c r="J64" s="1" t="s">
         <v>144</v>
@@ -3559,77 +3559,89 @@
     </row>
     <row r="65" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A65" s="1">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B65" s="1" t="s">
         <v>107</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>274</v>
+        <v>114</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="H65" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="I65" s="1" t="s">
         <v>272</v>
       </c>
-      <c r="I65" s="1" t="s">
-        <v>273</v>
-      </c>
       <c r="J65" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="N65" s="1" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="66" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A66" s="1">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>107</v>
+        <v>84</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="D66" s="1" t="s">
-        <v>121</v>
+        <v>203</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>283</v>
+        <v>327</v>
+      </c>
+      <c r="G66" s="1" t="s">
+        <v>144</v>
       </c>
       <c r="H66" s="1" t="s">
-        <v>272</v>
+        <v>229</v>
       </c>
       <c r="I66" s="1" t="s">
-        <v>273</v>
+        <v>229</v>
       </c>
       <c r="J66" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="N66" s="1" t="s">
-        <v>144</v>
+        <v>229</v>
+      </c>
+      <c r="K66" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="L66" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="M66" s="1" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="67" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A67" s="1">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B67" s="1" t="s">
         <v>84</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>204</v>
+        <v>87</v>
+      </c>
+      <c r="D67" s="1" t="s">
+        <v>91</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F67" s="1" t="s">
         <v>317</v>
@@ -3638,236 +3650,236 @@
         <v>144</v>
       </c>
       <c r="H67" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I67" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="J67" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="K67" s="1" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="L67" s="1" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="M67" s="1" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="68" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A68" s="1">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B68" s="1" t="s">
         <v>84</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="D68" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="E68" s="1" t="s">
-        <v>279</v>
+        <v>316</v>
+      </c>
+      <c r="D68" s="2"/>
+      <c r="E68" s="2" t="s">
+        <v>278</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="G68" s="1" t="s">
         <v>144</v>
       </c>
       <c r="H68" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I68" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="J68" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="K68" s="1" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="L68" s="1" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="M68" s="1" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="69" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="69" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A69" s="1">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B69" s="1" t="s">
         <v>84</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>318</v>
-      </c>
-      <c r="D69" s="2"/>
-      <c r="E69" s="2" t="s">
-        <v>279</v>
+        <v>85</v>
+      </c>
+      <c r="D69" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="E69" s="1" t="s">
+        <v>278</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>319</v>
-      </c>
-      <c r="G69" s="1" t="s">
-        <v>144</v>
+        <v>281</v>
       </c>
       <c r="H69" s="1" t="s">
-        <v>230</v>
+        <v>271</v>
       </c>
       <c r="I69" s="1" t="s">
-        <v>230</v>
+        <v>272</v>
       </c>
       <c r="J69" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="K69" s="1" t="s">
-        <v>244</v>
-      </c>
-      <c r="L69" s="1" t="s">
-        <v>233</v>
-      </c>
-      <c r="M69" s="1" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="70" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="70" spans="1:14" ht="72" x14ac:dyDescent="0.3">
       <c r="A70" s="1">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B70" s="1" t="s">
         <v>84</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F70" s="1" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="H70" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="I70" s="1" t="s">
         <v>272</v>
       </c>
-      <c r="I70" s="1" t="s">
-        <v>273</v>
-      </c>
       <c r="J70" s="1" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="71" spans="1:14" ht="72" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:14" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A71" s="1">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B71" s="1" t="s">
         <v>84</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F71" s="1" t="s">
         <v>283</v>
       </c>
       <c r="H71" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="I71" s="1" t="s">
         <v>272</v>
       </c>
-      <c r="I71" s="1" t="s">
-        <v>273</v>
-      </c>
       <c r="J71" s="1" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="72" spans="1:14" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A72" s="1">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B72" s="1" t="s">
         <v>84</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="D72" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="E72" s="1" t="s">
-        <v>279</v>
+        <v>94</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E72" s="2" t="s">
+        <v>278</v>
       </c>
       <c r="F72" s="1" t="s">
         <v>283</v>
       </c>
+      <c r="G72" s="2"/>
       <c r="H72" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="I72" s="1" t="s">
         <v>272</v>
       </c>
-      <c r="I72" s="1" t="s">
-        <v>273</v>
-      </c>
       <c r="J72" s="1" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="73" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A73" s="1">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>84</v>
+        <v>215</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="D73" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="E73" s="2" t="s">
-        <v>279</v>
+        <v>219</v>
+      </c>
+      <c r="D73" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E73" s="1" t="s">
+        <v>278</v>
       </c>
       <c r="F73" s="1" t="s">
-        <v>283</v>
-      </c>
-      <c r="G73" s="2"/>
+        <v>287</v>
+      </c>
+      <c r="G73" s="1" t="s">
+        <v>144</v>
+      </c>
       <c r="H73" s="1" t="s">
-        <v>272</v>
+        <v>229</v>
       </c>
       <c r="I73" s="1" t="s">
-        <v>273</v>
+        <v>229</v>
       </c>
       <c r="J73" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="K73" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="L73" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="M73" s="1" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="74" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A74" s="1">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C74" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="D74" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="D74" s="1" t="s">
-        <v>218</v>
-      </c>
       <c r="E74" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F74" s="1" t="s">
         <v>288</v>
@@ -3876,16 +3888,16 @@
         <v>144</v>
       </c>
       <c r="H74" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I74" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="J74" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="K74" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="L74" s="1" t="s">
         <v>144</v>
@@ -3896,106 +3908,103 @@
     </row>
     <row r="75" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A75" s="1">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B75" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="C75" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="D75" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="C75" s="1" t="s">
-        <v>222</v>
-      </c>
-      <c r="D75" s="1" t="s">
-        <v>221</v>
-      </c>
       <c r="E75" s="1" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="F75" s="1" t="s">
-        <v>289</v>
-      </c>
-      <c r="G75" s="1" t="s">
-        <v>144</v>
+        <v>281</v>
       </c>
       <c r="H75" s="1" t="s">
-        <v>230</v>
+        <v>144</v>
       </c>
       <c r="I75" s="1" t="s">
-        <v>230</v>
+        <v>144</v>
       </c>
       <c r="J75" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="K75" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="L75" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="M75" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="76" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="76" spans="1:14" ht="345.6" x14ac:dyDescent="0.3">
       <c r="A76" s="1">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>216</v>
+        <v>78</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>219</v>
+        <v>79</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>217</v>
+        <v>80</v>
       </c>
       <c r="E76" s="1" t="s">
         <v>278</v>
       </c>
       <c r="F76" s="1" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="H76" s="1" t="s">
-        <v>144</v>
+        <v>269</v>
       </c>
       <c r="I76" s="1" t="s">
-        <v>144</v>
+        <v>270</v>
       </c>
       <c r="J76" s="1" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="77" spans="1:14" ht="345.6" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A77" s="1">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B77" s="1" t="s">
         <v>78</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="D77" s="1" t="s">
-        <v>80</v>
+        <v>201</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F77" s="1" t="s">
-        <v>285</v>
+        <v>301</v>
+      </c>
+      <c r="G77" s="1" t="s">
+        <v>144</v>
       </c>
       <c r="H77" s="1" t="s">
-        <v>270</v>
+        <v>229</v>
       </c>
       <c r="I77" s="1" t="s">
-        <v>271</v>
+        <v>229</v>
       </c>
       <c r="J77" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="78" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+        <v>229</v>
+      </c>
+      <c r="K77" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="L77" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="M77" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="78" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A78" s="1">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B78" s="1" t="s">
         <v>78</v>
@@ -4004,229 +4013,220 @@
         <v>202</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F78" s="1" t="s">
-        <v>302</v>
+        <v>318</v>
       </c>
       <c r="G78" s="1" t="s">
         <v>144</v>
       </c>
       <c r="H78" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I78" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="J78" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="K78" s="1" t="s">
         <v>244</v>
       </c>
       <c r="L78" s="1" t="s">
-        <v>233</v>
+        <v>244</v>
       </c>
       <c r="M78" s="1" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="79" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="79" spans="1:14" ht="374.4" x14ac:dyDescent="0.3">
       <c r="A79" s="1">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B79" s="1" t="s">
         <v>78</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>203</v>
+        <v>81</v>
+      </c>
+      <c r="D79" s="1" t="s">
+        <v>82</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F79" s="1" t="s">
-        <v>320</v>
-      </c>
-      <c r="G79" s="1" t="s">
-        <v>144</v>
+        <v>282</v>
       </c>
       <c r="H79" s="1" t="s">
-        <v>230</v>
+        <v>271</v>
       </c>
       <c r="I79" s="1" t="s">
-        <v>230</v>
+        <v>270</v>
       </c>
       <c r="J79" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="K79" s="1" t="s">
-        <v>245</v>
-      </c>
-      <c r="L79" s="1" t="s">
-        <v>245</v>
-      </c>
-      <c r="M79" s="1" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="80" spans="1:14" ht="374.4" x14ac:dyDescent="0.3">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="80" spans="1:14" ht="273.60000000000002" x14ac:dyDescent="0.3">
       <c r="A80" s="1">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B80" s="1" t="s">
         <v>78</v>
       </c>
       <c r="C80" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="D80" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E80" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="F80" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="H80" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="I80" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="J80" s="1" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="81" spans="1:13" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A81" s="1">
         <v>81</v>
       </c>
-      <c r="D80" s="1" t="s">
+      <c r="B81" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C81" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D81" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="E81" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="F81" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="G81" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="H81" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="I81" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="J81" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="K81" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="L81" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="M81" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="82" spans="1:13" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A82" s="1">
         <v>82</v>
-      </c>
-      <c r="E80" s="1" t="s">
-        <v>279</v>
-      </c>
-      <c r="F80" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="H80" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="I80" s="1" t="s">
-        <v>271</v>
-      </c>
-      <c r="J80" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="81" spans="1:13" ht="273.60000000000002" x14ac:dyDescent="0.3">
-      <c r="A81" s="1">
-        <v>80</v>
-      </c>
-      <c r="B81" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="C81" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="D81" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="E81" s="1" t="s">
-        <v>279</v>
-      </c>
-      <c r="F81" s="1" t="s">
-        <v>283</v>
-      </c>
-      <c r="H81" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="I81" s="1" t="s">
-        <v>273</v>
-      </c>
-      <c r="J81" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="82" spans="1:13" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A82" s="1">
-        <v>81</v>
       </c>
       <c r="B82" s="1" t="s">
         <v>38</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>40</v>
+        <v>145</v>
       </c>
       <c r="D82" s="1" t="s">
         <v>237</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F82" s="1" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="G82" s="1" t="s">
-        <v>144</v>
+        <v>319</v>
       </c>
       <c r="H82" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I82" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="J82" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="K82" s="1" t="s">
         <v>144</v>
       </c>
       <c r="L82" s="1" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="M82" s="1" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="83" spans="1:13" ht="57.6" x14ac:dyDescent="0.3">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="83" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A83" s="1">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B83" s="1" t="s">
         <v>38</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="D83" s="1" t="s">
-        <v>238</v>
+        <v>194</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F83" s="1" t="s">
-        <v>296</v>
-      </c>
-      <c r="G83" s="1" t="s">
-        <v>321</v>
+        <v>282</v>
       </c>
       <c r="H83" s="1" t="s">
         <v>230</v>
       </c>
       <c r="I83" s="1" t="s">
-        <v>230</v>
+        <v>144</v>
       </c>
       <c r="J83" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="K83" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="L83" s="1" t="s">
-        <v>233</v>
-      </c>
-      <c r="M83" s="1" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="84" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="84" spans="1:13" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A84" s="1">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B84" s="1" t="s">
         <v>38</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>195</v>
+        <v>39</v>
+      </c>
+      <c r="D84" s="1" t="s">
+        <v>67</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F84" s="1" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="H84" s="1" t="s">
-        <v>231</v>
+        <v>144</v>
       </c>
       <c r="I84" s="1" t="s">
         <v>144</v>
@@ -4235,59 +4235,65 @@
         <v>144</v>
       </c>
     </row>
-    <row r="85" spans="1:13" ht="158.4" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A85" s="1">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D85" s="1" t="s">
-        <v>67</v>
+        <v>46</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F85" s="1" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="H85" s="1" t="s">
-        <v>144</v>
+        <v>229</v>
       </c>
       <c r="I85" s="1" t="s">
-        <v>144</v>
+        <v>229</v>
       </c>
       <c r="J85" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="K85" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="L85" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="M85" s="1" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="86" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A86" s="1">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B86" s="1" t="s">
         <v>25</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>46</v>
+        <v>4</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F86" s="1" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="H86" s="1" t="s">
-        <v>230</v>
+        <v>266</v>
       </c>
       <c r="I86" s="1" t="s">
-        <v>230</v>
+        <v>144</v>
       </c>
       <c r="J86" s="1" t="s">
-        <v>230</v>
+        <v>144</v>
       </c>
       <c r="K86" s="1" t="s">
         <v>144</v>
@@ -4301,22 +4307,22 @@
     </row>
     <row r="87" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A87" s="1">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B87" s="1" t="s">
         <v>25</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F87" s="1" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="H87" s="1" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="I87" s="1" t="s">
         <v>144</v>
@@ -4334,24 +4340,24 @@
         <v>144</v>
       </c>
     </row>
-    <row r="88" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A88" s="1">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B88" s="1" t="s">
         <v>25</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E88" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F88" s="1" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="H88" s="1" t="s">
-        <v>267</v>
+        <v>144</v>
       </c>
       <c r="I88" s="1" t="s">
         <v>144</v>
@@ -4371,19 +4377,19 @@
     </row>
     <row r="89" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A89" s="1">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B89" s="1" t="s">
         <v>25</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F89" s="1" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="H89" s="1" t="s">
         <v>144</v>
@@ -4406,19 +4412,19 @@
     </row>
     <row r="90" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A90" s="1">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B90" s="1" t="s">
         <v>25</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>3</v>
+        <v>131</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F90" s="1" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="H90" s="1" t="s">
         <v>144</v>
@@ -4439,21 +4445,24 @@
         <v>144</v>
       </c>
     </row>
-    <row r="91" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:13" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A91" s="1">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B91" s="1" t="s">
         <v>25</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>131</v>
+        <v>189</v>
+      </c>
+      <c r="D91" s="1" t="s">
+        <v>190</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F91" s="1" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="H91" s="1" t="s">
         <v>144</v>
@@ -4464,34 +4473,22 @@
       <c r="J91" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="K91" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="L91" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="M91" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="92" spans="1:13" ht="43.2" x14ac:dyDescent="0.3">
+    </row>
+    <row r="92" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A92" s="1">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>25</v>
+        <v>187</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="D92" s="1" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F92" s="1" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="H92" s="1" t="s">
         <v>144</v>
@@ -4503,35 +4500,47 @@
         <v>144</v>
       </c>
     </row>
-    <row r="93" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:13" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A93" s="1">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>188</v>
+        <v>125</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>189</v>
+        <v>211</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F93" s="1" t="s">
-        <v>282</v>
+        <v>320</v>
+      </c>
+      <c r="G93" s="1" t="s">
+        <v>144</v>
       </c>
       <c r="H93" s="1" t="s">
-        <v>144</v>
+        <v>229</v>
       </c>
       <c r="I93" s="1" t="s">
-        <v>144</v>
+        <v>229</v>
       </c>
       <c r="J93" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="94" spans="1:13" ht="100.8" x14ac:dyDescent="0.3">
+        <v>229</v>
+      </c>
+      <c r="K93" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="L93" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="M93" s="1" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="94" spans="1:13" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A94" s="1">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B94" s="1" t="s">
         <v>125</v>
@@ -4540,130 +4549,121 @@
         <v>212</v>
       </c>
       <c r="E94" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F94" s="1" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="G94" s="1" t="s">
         <v>144</v>
       </c>
       <c r="H94" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I94" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="J94" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="K94" s="1" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="L94" s="1" t="s">
-        <v>262</v>
+        <v>144</v>
       </c>
       <c r="M94" s="1" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="95" spans="1:13" ht="57.6" x14ac:dyDescent="0.3">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="95" spans="1:13" ht="72" x14ac:dyDescent="0.3">
       <c r="A95" s="1">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B95" s="1" t="s">
         <v>125</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>213</v>
+        <v>138</v>
+      </c>
+      <c r="D95" s="1" t="s">
+        <v>140</v>
       </c>
       <c r="E95" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F95" s="1" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="G95" s="1" t="s">
         <v>144</v>
       </c>
       <c r="H95" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I95" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="J95" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="K95" s="1" t="s">
         <v>263</v>
       </c>
       <c r="L95" s="1" t="s">
-        <v>144</v>
+        <v>264</v>
       </c>
       <c r="M95" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="96" spans="1:13" ht="72" x14ac:dyDescent="0.3">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="96" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A96" s="1">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B96" s="1" t="s">
         <v>125</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="D96" s="1" t="s">
-        <v>140</v>
+        <v>127</v>
       </c>
       <c r="E96" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F96" s="1" t="s">
-        <v>324</v>
-      </c>
-      <c r="G96" s="1" t="s">
-        <v>144</v>
+        <v>281</v>
       </c>
       <c r="H96" s="1" t="s">
-        <v>230</v>
+        <v>144</v>
       </c>
       <c r="I96" s="1" t="s">
-        <v>230</v>
+        <v>144</v>
       </c>
       <c r="J96" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="K96" s="1" t="s">
-        <v>264</v>
-      </c>
-      <c r="L96" s="1" t="s">
-        <v>265</v>
-      </c>
-      <c r="M96" s="1" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="97" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="97" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A97" s="1">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B97" s="1" t="s">
         <v>125</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="D97" s="1" t="s">
-        <v>127</v>
+        <v>150</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F97" s="1" t="s">
-        <v>282</v>
+        <v>323</v>
       </c>
       <c r="H97" s="1" t="s">
         <v>144</v>
@@ -4674,25 +4674,25 @@
       <c r="J97" s="1" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="98" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="K97" s="1" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="98" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A98" s="1">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B98" s="1" t="s">
         <v>125</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="D98" s="1" t="s">
-        <v>151</v>
+        <v>136</v>
       </c>
       <c r="E98" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F98" s="1" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="H98" s="1" t="s">
         <v>144</v>
@@ -4701,27 +4701,27 @@
         <v>144</v>
       </c>
       <c r="J98" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="K98" s="1" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="99" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A99" s="1">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B99" s="1" t="s">
         <v>125</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
+      </c>
+      <c r="D99" s="1" t="s">
+        <v>213</v>
       </c>
       <c r="E99" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F99" s="1" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="H99" s="1" t="s">
         <v>144</v>
@@ -4735,22 +4735,22 @@
     </row>
     <row r="100" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A100" s="1">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B100" s="1" t="s">
         <v>125</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D100" s="1" t="s">
         <v>214</v>
       </c>
       <c r="E100" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F100" s="1" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="H100" s="1" t="s">
         <v>144</v>
@@ -4762,216 +4762,213 @@
         <v>144</v>
       </c>
     </row>
-    <row r="101" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A101" s="1">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B101" s="1" t="s">
         <v>125</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D101" s="1" t="s">
-        <v>215</v>
+        <v>142</v>
       </c>
       <c r="E101" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F101" s="1" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="H101" s="1" t="s">
-        <v>144</v>
+        <v>265</v>
       </c>
       <c r="I101" s="1" t="s">
-        <v>144</v>
+        <v>265</v>
       </c>
       <c r="J101" s="1" t="s">
-        <v>144</v>
+        <v>265</v>
       </c>
     </row>
     <row r="102" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A102" s="1">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B102" s="1" t="s">
         <v>125</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="D102" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E102" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F102" s="1" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="H102" s="1" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="I102" s="1" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="J102" s="1" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="103" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="103" spans="1:14" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A103" s="1">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B103" s="1" t="s">
         <v>125</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>143</v>
+        <v>128</v>
+      </c>
+      <c r="D103" s="1" t="s">
+        <v>134</v>
       </c>
       <c r="E103" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F103" s="1" t="s">
-        <v>327</v>
+        <v>282</v>
       </c>
       <c r="H103" s="1" t="s">
-        <v>266</v>
+        <v>256</v>
       </c>
       <c r="I103" s="1" t="s">
-        <v>266</v>
+        <v>256</v>
       </c>
       <c r="J103" s="1" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="104" spans="1:14" ht="86.4" x14ac:dyDescent="0.3">
+        <v>256</v>
+      </c>
+      <c r="K103" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="L103" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="M103" s="1" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="104" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A104" s="1">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B104" s="1" t="s">
         <v>125</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D104" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E104" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F104" s="1" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="H104" s="1" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="I104" s="1" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="J104" s="1" t="s">
-        <v>257</v>
-      </c>
-      <c r="K104" s="1" t="s">
-        <v>258</v>
-      </c>
-      <c r="L104" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="M104" s="1" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="105" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="105" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A105" s="1">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="D105" s="1" t="s">
-        <v>135</v>
+        <v>210</v>
       </c>
       <c r="E105" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F105" s="1" t="s">
-        <v>283</v>
+        <v>294</v>
+      </c>
+      <c r="G105" s="1" t="s">
+        <v>298</v>
       </c>
       <c r="H105" s="1" t="s">
-        <v>260</v>
+        <v>229</v>
       </c>
       <c r="I105" s="1" t="s">
-        <v>260</v>
+        <v>229</v>
       </c>
       <c r="J105" s="1" t="s">
-        <v>260</v>
+        <v>229</v>
+      </c>
+      <c r="K105" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="L105" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="M105" s="1" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="106" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A106" s="1">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B106" s="1" t="s">
         <v>132</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="D106" s="1" t="s">
-        <v>211</v>
+        <v>174</v>
       </c>
       <c r="E106" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F106" s="1" t="s">
-        <v>295</v>
-      </c>
-      <c r="G106" s="1" t="s">
-        <v>299</v>
+        <v>282</v>
       </c>
       <c r="H106" s="1" t="s">
         <v>230</v>
       </c>
       <c r="I106" s="1" t="s">
-        <v>230</v>
+        <v>144</v>
       </c>
       <c r="J106" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="K106" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="L106" s="1" t="s">
-        <v>233</v>
-      </c>
-      <c r="M106" s="1" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="107" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="107" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A107" s="1">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B107" s="1" t="s">
         <v>132</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E107" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F107" s="1" t="s">
-        <v>283</v>
+        <v>323</v>
       </c>
       <c r="H107" s="1" t="s">
-        <v>231</v>
+        <v>144</v>
       </c>
       <c r="I107" s="1" t="s">
         <v>144</v>
@@ -4982,19 +4979,19 @@
     </row>
     <row r="108" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A108" s="1">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>132</v>
+        <v>181</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="E108" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F108" s="1" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="H108" s="1" t="s">
         <v>144</v>
@@ -5006,21 +5003,21 @@
         <v>144</v>
       </c>
     </row>
-    <row r="109" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A109" s="1">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="C109" s="1" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="E109" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F109" s="1" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="H109" s="1" t="s">
         <v>144</v>
@@ -5032,21 +5029,21 @@
         <v>144</v>
       </c>
     </row>
-    <row r="110" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A110" s="1">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="C110" s="1" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="E110" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F110" s="1" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="H110" s="1" t="s">
         <v>144</v>
@@ -5057,22 +5054,25 @@
       <c r="J110" s="1" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="111" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="N110" s="1" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="111" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A111" s="1">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="C111" s="1" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="E111" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F111" s="1" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="H111" s="1" t="s">
         <v>144</v>
@@ -5083,144 +5083,115 @@
       <c r="J111" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="N111" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="112" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="112" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A112" s="1">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>176</v>
+        <v>28</v>
       </c>
       <c r="C112" s="1" t="s">
-        <v>177</v>
+        <v>31</v>
       </c>
       <c r="E112" s="1" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="F112" s="1" t="s">
-        <v>325</v>
+        <v>326</v>
+      </c>
+      <c r="G112" s="1" t="s">
+        <v>144</v>
       </c>
       <c r="H112" s="1" t="s">
-        <v>144</v>
+        <v>229</v>
       </c>
       <c r="I112" s="1" t="s">
-        <v>144</v>
+        <v>229</v>
       </c>
       <c r="J112" s="1" t="s">
-        <v>144</v>
+        <v>229</v>
+      </c>
+      <c r="K112" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="L112" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="M112" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="N112" s="1" t="s">
+        <v>230</v>
       </c>
     </row>
     <row r="113" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A113" s="1">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B113" s="1" t="s">
         <v>28</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E113" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F113" s="1" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="G113" s="1" t="s">
         <v>144</v>
       </c>
       <c r="H113" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="I113" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="J113" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="K113" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="L113" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="M113" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="N113" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="I113" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="J113" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="K113" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="L113" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="M113" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="N113" s="1" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="114" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+    </row>
+    <row r="114" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A114" s="1">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B114" s="1" t="s">
         <v>28</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E114" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F114" s="1" t="s">
-        <v>328</v>
-      </c>
-      <c r="G114" s="1" t="s">
-        <v>144</v>
+        <v>283</v>
       </c>
       <c r="H114" s="1" t="s">
-        <v>230</v>
+        <v>144</v>
       </c>
       <c r="I114" s="1" t="s">
-        <v>230</v>
+        <v>144</v>
       </c>
       <c r="J114" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="K114" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="L114" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="M114" s="1" t="s">
         <v>144</v>
       </c>
       <c r="N114" s="1" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="115" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A115" s="1">
-        <v>114</v>
-      </c>
-      <c r="B115" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C115" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E115" s="1" t="s">
-        <v>279</v>
-      </c>
-      <c r="F115" s="1" t="s">
-        <v>284</v>
-      </c>
-      <c r="H115" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="I115" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="J115" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="N115" s="1" t="s">
         <v>144</v>
       </c>
     </row>
@@ -5295,16 +5266,16 @@
         <v>18</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>153</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>154</v>
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
@@ -5314,16 +5285,16 @@
         <v>21</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>166</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>167</v>
       </c>
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
@@ -5344,16 +5315,16 @@
         <v>22</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="E7" s="1" t="s">
         <v>162</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>163</v>
       </c>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
@@ -5363,16 +5334,16 @@
         <v>23</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="E8" s="1" t="s">
         <v>158</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>159</v>
       </c>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
@@ -5382,16 +5353,16 @@
         <v>24</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="E9" s="1" t="s">
         <v>170</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>171</v>
       </c>
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
@@ -5401,11 +5372,11 @@
         <v>132</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C10" s="1"/>
       <c r="D10" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>

</xml_diff>